<commit_message>
feat(fase-1): logo AA Montagens vetorizada em SVG
- logo-full / logo-mono / logo-simbolo: 489 nos, 15 paths nomeados
- perda de fidelidade zero (IoU no teto do raster: 0.9729 azul / 0.9433 preto)
- svgo em modo absoluto, IoU otimizado vs bruto = 1.00000, ids preservados
- paleta extraida: #135885 azul-aco, #1C1A17 preto quente, #E8E4DF bege osso
- tools/: tracador proprio (crack following + RDP) e conferidor por IoU
- docs/decisoes.md: D1..D9 das respostas da Fase 0

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IGREJA SAO MIGUEL ARCANJO PORTA PEROLA 2.xlsx
+++ b/IGREJA SAO MIGUEL ARCANJO PORTA PEROLA 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\AA MONTAGENS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/39afe70b92a45968/Área de Trabalho/roberta/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{7435C746-FF92-44B9-A455-7F530904AA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ORÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -637,53 +637,53 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1037,9 +1037,9 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.109375" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
     <col min="3" max="4" width="9" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
@@ -1047,195 +1047,195 @@
     <col min="7" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="40"/>
-      <c r="B1" s="40"/>
-      <c r="C1" s="49" t="s">
+    <row r="1" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="46"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="40"/>
-      <c r="B2" s="40"/>
-      <c r="C2" s="39" t="s">
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="46"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-    </row>
-    <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40"/>
-      <c r="B3" s="40"/>
-      <c r="C3" s="39" t="s">
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+    </row>
+    <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-    </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="40"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="39" t="s">
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+    </row>
+    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="46"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
-    </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="40"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="39" t="s">
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+    </row>
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="46"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-    </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="40"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="39" t="s">
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="46"/>
+    </row>
+    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="46"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-    </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="40"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="40"/>
-    </row>
-    <row r="8" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="50" t="s">
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
+    </row>
+    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="46"/>
+      <c r="B7" s="46"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="46"/>
+    </row>
+    <row r="8" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="50"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="50"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="50"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="50"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="50"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="50"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="48"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="48"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="52"/>
-      <c r="D10" s="52"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
       <c r="E10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="51">
+      <c r="F10" s="50">
         <v>46248</v>
       </c>
-      <c r="G10" s="52"/>
-      <c r="H10" s="52"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="53"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
       <c r="E11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="53"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F11" s="36"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="53"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B12" s="36"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="53"/>
-      <c r="C13" s="52"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="37"/>
       <c r="D13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="53"/>
+      <c r="E13" s="36"/>
       <c r="F13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="53"/>
-      <c r="H13" s="52"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G13" s="36"/>
+      <c r="H13" s="37"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="53"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="52"/>
-      <c r="G14" s="52"/>
-      <c r="H14" s="52"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B14" s="36"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="53"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="52"/>
-      <c r="H15" s="52"/>
-    </row>
-    <row r="16" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="36"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+    </row>
+    <row r="16" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
@@ -1255,7 +1255,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>1</v>
       </c>
@@ -1267,7 +1267,7 @@
       <c r="E17" s="30"/>
       <c r="F17" s="30"/>
     </row>
-    <row r="18" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>43</v>
       </c>
@@ -1280,15 +1280,15 @@
       <c r="D18" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="37">
+      <c r="E18" s="52">
         <v>25600</v>
       </c>
-      <c r="F18" s="38">
+      <c r="F18" s="53">
         <f t="shared" ref="F18:F27" si="0">IF(OR(C18="",E18=""),"",C18*E18)</f>
         <v>25600</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>44</v>
       </c>
@@ -1301,10 +1301,10 @@
       <c r="D19" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="37"/>
-      <c r="F19" s="38"/>
-    </row>
-    <row r="20" spans="1:8" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E19" s="52"/>
+      <c r="F19" s="53"/>
+    </row>
+    <row r="20" spans="1:8" ht="52.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>45</v>
       </c>
@@ -1317,10 +1317,10 @@
       <c r="D20" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="37"/>
-      <c r="F20" s="38"/>
-    </row>
-    <row r="21" spans="1:8" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E20" s="52"/>
+      <c r="F20" s="53"/>
+    </row>
+    <row r="21" spans="1:8" ht="43.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
         <v>46</v>
       </c>
@@ -1333,10 +1333,10 @@
       <c r="D21" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="37"/>
-      <c r="F21" s="38"/>
-    </row>
-    <row r="22" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E21" s="52"/>
+      <c r="F21" s="53"/>
+    </row>
+    <row r="22" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="str">
         <f>IF(OR(C22="",E22=""),"",C22*E22)</f>
         <v/>
@@ -1347,7 +1347,7 @@
       <c r="E22" s="23"/>
       <c r="F22" s="15"/>
     </row>
-    <row r="23" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="24">
         <v>2</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
         <v>49</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>51</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" s="31"/>
       <c r="C26" s="26"/>
@@ -1403,7 +1403,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="17"/>
       <c r="C27" s="16"/>
@@ -1414,54 +1414,54 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="44" t="s">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="43"/>
+      <c r="B28" s="41"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="42"/>
       <c r="F28" s="4">
         <f>SUM(F18:F27)</f>
         <v>25600</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="47" t="s">
+    <row r="29" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="40"/>
-      <c r="C29" s="40"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
-    </row>
-    <row r="30" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="47"/>
-      <c r="B30" s="40"/>
-      <c r="C30" s="40"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="40"/>
-      <c r="F30" s="40"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="48" t="s">
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+    </row>
+    <row r="30" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="45"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="40"/>
-      <c r="C31" s="40"/>
-      <c r="D31" s="40"/>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40"/>
-    </row>
-    <row r="32" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="41" t="s">
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+    </row>
+    <row r="32" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="B32" s="42"/>
-      <c r="C32" s="42"/>
-      <c r="D32" s="43"/>
+      <c r="B32" s="41"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="42"/>
       <c r="E32" s="5" t="s">
         <v>21</v>
       </c>
@@ -1469,30 +1469,30 @@
         <f>F28</f>
         <v>25600</v>
       </c>
-      <c r="G32" s="45"/>
-      <c r="H32" s="45"/>
-    </row>
-    <row r="33" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="56" t="s">
+      <c r="G32" s="43"/>
+      <c r="H32" s="43"/>
+    </row>
+    <row r="33" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="43"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="42"/>
       <c r="E33" s="7" t="s">
         <v>26</v>
       </c>
       <c r="F33" s="8">
         <v>0</v>
       </c>
-      <c r="G33" s="45"/>
-      <c r="H33" s="45"/>
-    </row>
-    <row r="34" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="57"/>
-      <c r="B34" s="42"/>
-      <c r="C34" s="42"/>
-      <c r="D34" s="43"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="43"/>
+    </row>
+    <row r="34" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="44"/>
+      <c r="B34" s="41"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="42"/>
       <c r="E34" s="7" t="s">
         <v>27</v>
       </c>
@@ -1500,67 +1500,74 @@
         <f>F32+F33</f>
         <v>25600</v>
       </c>
-      <c r="G34" s="45"/>
-      <c r="H34" s="45"/>
-    </row>
-    <row r="35" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="46" t="s">
+      <c r="G34" s="43"/>
+      <c r="H34" s="43"/>
+    </row>
+    <row r="35" spans="1:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="42"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="43"/>
+      <c r="B35" s="41"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="42"/>
       <c r="E35" s="5" t="s">
         <v>28</v>
       </c>
       <c r="F35" s="10">
         <v>0</v>
       </c>
-      <c r="G35" s="55" t="s">
+      <c r="G35" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="H35" s="54">
+      <c r="H35" s="38">
         <f>F34-F35</f>
         <v>25600</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="36" t="s">
+    <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="51" t="s">
         <v>30</v>
       </c>
-      <c r="B37" s="40"/>
-      <c r="C37" s="40"/>
-      <c r="E37" s="36" t="s">
+      <c r="B37" s="46"/>
+      <c r="C37" s="46"/>
+      <c r="E37" s="51" t="s">
         <v>30</v>
       </c>
-      <c r="F37" s="40"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="40"/>
-    </row>
-    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="36" t="s">
+      <c r="F37" s="46"/>
+      <c r="G37" s="46"/>
+      <c r="H37" s="46"/>
+    </row>
+    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B38" s="36"/>
-      <c r="E38" s="36" t="s">
+      <c r="B38" s="51"/>
+      <c r="E38" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
-    </row>
-    <row r="39" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="F38" s="51"/>
+      <c r="G38" s="51"/>
+    </row>
+    <row r="39" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="F11:H11"/>
-    <mergeCell ref="H35"/>
-    <mergeCell ref="G35"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="H32"/>
-    <mergeCell ref="G34"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="E37:H37"/>
+    <mergeCell ref="G33"/>
+    <mergeCell ref="H33"/>
+    <mergeCell ref="G32"/>
+    <mergeCell ref="H34"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="C1:H1"/>
     <mergeCell ref="A8:H9"/>
     <mergeCell ref="C6:H6"/>
@@ -1577,22 +1584,15 @@
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="E13"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="E37:H37"/>
-    <mergeCell ref="G33"/>
-    <mergeCell ref="H33"/>
-    <mergeCell ref="G32"/>
-    <mergeCell ref="H34"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="H35"/>
+    <mergeCell ref="G35"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="H32"/>
+    <mergeCell ref="G34"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A29:F29"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup paperSize="9" scale="72" orientation="portrait" r:id="rId1"/>
@@ -1607,37 +1607,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>37</v>
       </c>

</xml_diff>